<commit_message>
Stat sheet: add Teiko and Equinox rosters (now 161 players, 12 teams)
Append the Teiko (11 players, ASIA/OCE) and Equinox (15 players, ASIA)
registrations to the Stats tab and give each its own roster tab.
Teiko's joke position spellings (sitter / midol bloker / ol rownder /
awtsayd / upusit / lebero) are normalized to the standard names.
</commit_message>
<xml_diff>
--- a/files/binsu-stat-sheet.xlsx
+++ b/files/binsu-stat-sheet.xlsx
@@ -18,7 +18,9 @@
     <sheet name="Orchid" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="The Order" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Kittyoo" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Instructions" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Teiko" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Equinox" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Instructions" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -513,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5710,15 +5712,1003 @@
         <v>0</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>LB_Tempted</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="138">
-      <c r="A138" s="6" t="inlineStr">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>zimon25</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>Choiixzn</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>RisingBlades</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>rehaniv12</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Ace_Ish1kawa</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Opposite</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>DarkEclips_e</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>AnkaaMGL0804</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>gwagwacattroll</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>Libero</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>TW_Jupiter</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>DominuzGrey</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>RoyaleMice6</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Setter/All-Rounder</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>memenoob345</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>Outside/All-Rounder</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>sulhipip</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Opposite</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>kouuuuuuw</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>KungKangg</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Libero</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>Gelatinousious</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/All-Rounder</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>GGgrazyGG</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Libero/Middle</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>NABILGOTMELIKE</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Setter/Libero</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Pazzel</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Setter</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>vex</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>lwkeyfinn</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Outside</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>DarkJackxx12</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Outside</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>tadatsuneshinkai</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>kenderdragoonca74</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>llewor1234</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="inlineStr">
         <is>
           <t>Every registered player is pre-filled — just update the numbers after each game (season totals). Add new signings as new rows.</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="6" t="inlineStr">
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
         <is>
           <t>Row 1 headers become the website's columns and leaderboard categories — don't rename them mid-season.</t>
         </is>
@@ -6691,6 +7681,862 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Region:</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>ASIA/OCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Captain:</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>RisingBlades (@risingblades)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Vice Captain:</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Choiixzn (@tsoii)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Players:</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Roblox username</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>LB_Tempted</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>@Jha</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>zimon25</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>@flam</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Choiixzn</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>@tsoii</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>RisingBlades</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>@risingblades</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>rehaniv12</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>@High cortisol</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Ace_Ish1kawa</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>@Lonely Guy</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Opposite</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DarkEclips_e</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>@DarkMoon</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>AnkaaMGL0804</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>@anando</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>gwagwacattroll</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>@bil</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Libero</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>TW_Jupiter</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>@Jupiter</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DominuzGrey</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>@greys</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Region:</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>ASIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Captain:</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>RoyaleMice6 (@!Frieza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Vice Captain:</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>memenoob345 (@nope)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Players:</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Roblox username</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>RoyaleMice6</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>@!Frieza</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Setter/All-Rounder</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>memenoob345</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>@nope</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Outside/All-Rounder</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>sulhipip</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>@jianxi1499</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Opposite</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>kouuuuuuw</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>@xiao</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>KungKangg</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>@KangKungg</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Libero</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Gelatinousious</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>@Tsundere Venir</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/All-Rounder</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GGgrazyGG</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>@Gray</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Libero/Middle</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>NABILGOTMELIKE</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>@Bilboe</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Setter/Libero</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Pazzel</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>@monz</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Setter</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>vex</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>@SØL</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>lwkeyfinn</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>@somebody</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Outside</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DarkJackxx12</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>@zenryu</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Outside</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>tadatsuneshinkai</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>@Drey</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>kenderdragoonca74</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>@Xinhdeplanhat</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>llewor1234</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>@russ</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Stat sheet: add Teiko and Equinox rosters (now 161 players, 12 teams) (#71)
Append the Teiko (11 players, ASIA/OCE) and Equinox (15 players, ASIA)
registrations to the Stats tab and give each its own roster tab.
Teiko's joke position spellings (sitter / midol bloker / ol rownder /
awtsayd / upusit / lebero) are normalized to the standard names.

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/binsu-stat-sheet.xlsx
+++ b/files/binsu-stat-sheet.xlsx
@@ -18,7 +18,9 @@
     <sheet name="Orchid" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="The Order" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Kittyoo" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Instructions" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Teiko" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Equinox" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Instructions" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -513,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J139"/>
+  <dimension ref="A1:J165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5710,15 +5712,1003 @@
         <v>0</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>LB_Tempted</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I137" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J137" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="138">
-      <c r="A138" s="6" t="inlineStr">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>zimon25</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I138" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J138" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="4" t="inlineStr">
+        <is>
+          <t>Choiixzn</t>
+        </is>
+      </c>
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I139" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J139" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>RisingBlades</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I140" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J140" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>rehaniv12</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I141" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J141" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>Ace_Ish1kawa</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Opposite</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I142" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J142" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>DarkEclips_e</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I143" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J143" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>AnkaaMGL0804</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I144" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J144" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="4" t="inlineStr">
+        <is>
+          <t>gwagwacattroll</t>
+        </is>
+      </c>
+      <c r="B145" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>Libero</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I145" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J145" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>TW_Jupiter</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I146" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J146" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="4" t="inlineStr">
+        <is>
+          <t>DominuzGrey</t>
+        </is>
+      </c>
+      <c r="B147" s="4" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I147" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J147" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>RoyaleMice6</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Setter/All-Rounder</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I148" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J148" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>memenoob345</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>Outside/All-Rounder</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I149" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J149" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>sulhipip</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Opposite</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>kouuuuuuw</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>KungKangg</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Libero</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>Gelatinousious</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/All-Rounder</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>GGgrazyGG</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Libero/Middle</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>NABILGOTMELIKE</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Setter/Libero</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Pazzel</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Setter</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I156" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J156" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>vex</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I157" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J157" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>lwkeyfinn</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Outside</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J158" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>DarkJackxx12</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Outside</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I159" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J159" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>tadatsuneshinkai</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I160" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J160" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>kenderdragoonca74</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I161" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J161" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>llewor1234</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I162" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J162" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="6" t="inlineStr">
         <is>
           <t>Every registered player is pre-filled — just update the numbers after each game (season totals). Add new signings as new rows.</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="6" t="inlineStr">
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
         <is>
           <t>Row 1 headers become the website's columns and leaderboard categories — don't rename them mid-season.</t>
         </is>
@@ -6691,6 +7681,862 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Teiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Region:</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>ASIA/OCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Captain:</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>RisingBlades (@risingblades)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Vice Captain:</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Choiixzn (@tsoii)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Players:</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Roblox username</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>LB_Tempted</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>@Jha</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>zimon25</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>@flam</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Choiixzn</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>@tsoii</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>RisingBlades</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>@risingblades</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>rehaniv12</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>@High cortisol</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Ace_Ish1kawa</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>@Lonely Guy</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Opposite</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>DarkEclips_e</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>@DarkMoon</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>All-Rounder</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>AnkaaMGL0804</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>@anando</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>gwagwacattroll</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>@bil</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Libero</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>TW_Jupiter</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>@Jupiter</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>DominuzGrey</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>@greys</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Setter</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Equinox</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Region:</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>ASIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Captain:</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>RoyaleMice6 (@!Frieza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Vice Captain:</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>memenoob345 (@nope)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Players:</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Roblox username</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Discord</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Squad</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>RoyaleMice6</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>@!Frieza</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Setter/All-Rounder</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>memenoob345</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>@nope</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Outside/All-Rounder</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>sulhipip</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>@jianxi1499</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Opposite</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>kouuuuuuw</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>@xiao</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Middle</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>KungKangg</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>@KangKungg</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Libero</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Gelatinousious</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>@Tsundere Venir</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/All-Rounder</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>GGgrazyGG</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>@Gray</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Libero/Middle</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>NABILGOTMELIKE</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>@Bilboe</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Setter/Libero</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Pazzel</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>@monz</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Outside/Setter</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>vex</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>@SØL</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>lwkeyfinn</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>@somebody</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Middle/Outside</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>DarkJackxx12</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>@zenryu</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Opposite/Outside</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>tadatsuneshinkai</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>@Drey</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>kenderdragoonca74</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>@Xinhdeplanhat</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Outside</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>llewor1234</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>@russ</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Opposite/Middle</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Sub</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>